<commit_message>
Continuing implementing 4 new tribes
</commit_message>
<xml_diff>
--- a/novas_tribos.xlsx
+++ b/novas_tribos.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Y:\www\t3\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\192.168.1.6\laragon\www\t3\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D31F3B5D-9470-4166-AD13-0A5DBD4B4F46}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31726B3C-EAEA-4D50-887A-49FAD3591142}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="288" yWindow="756" windowWidth="16080" windowHeight="17208" firstSheet="2" activeTab="5" xr2:uid="{A6F64B46-DD3A-4625-993E-1B49EC177123}"/>
+    <workbookView xWindow="1572" yWindow="9768" windowWidth="19392" windowHeight="12504" firstSheet="2" activeTab="6" xr2:uid="{A6F64B46-DD3A-4625-993E-1B49EC177123}"/>
   </bookViews>
   <sheets>
     <sheet name="unitdata" sheetId="1" r:id="rId1"/>
@@ -534,7 +534,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -546,15 +546,12 @@
     <xf numFmtId="46" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -19831,21 +19828,21 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="5"/>
-      <c r="C1" s="5"/>
-      <c r="D1" s="5"/>
-      <c r="E1" s="5"/>
-      <c r="F1" s="5"/>
-      <c r="G1" s="5"/>
-      <c r="H1" s="5"/>
-      <c r="I1" s="5"/>
-      <c r="J1" s="5"/>
-      <c r="K1" s="5"/>
-      <c r="L1" s="5"/>
-      <c r="M1" s="5"/>
+      <c r="B1" s="7"/>
+      <c r="C1" s="7"/>
+      <c r="D1" s="7"/>
+      <c r="E1" s="7"/>
+      <c r="F1" s="7"/>
+      <c r="G1" s="7"/>
+      <c r="H1" s="7"/>
+      <c r="I1" s="7"/>
+      <c r="J1" s="7"/>
+      <c r="K1" s="7"/>
+      <c r="L1" s="7"/>
+      <c r="M1" s="7"/>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
@@ -20299,21 +20296,21 @@
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A14" s="5" t="s">
+      <c r="A14" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="B14" s="5"/>
-      <c r="C14" s="5"/>
-      <c r="D14" s="5"/>
-      <c r="E14" s="5"/>
-      <c r="F14" s="5"/>
-      <c r="G14" s="5"/>
-      <c r="H14" s="5"/>
-      <c r="I14" s="5"/>
-      <c r="J14" s="5"/>
-      <c r="K14" s="5"/>
-      <c r="L14" s="5"/>
-      <c r="M14" s="5"/>
+      <c r="B14" s="7"/>
+      <c r="C14" s="7"/>
+      <c r="D14" s="7"/>
+      <c r="E14" s="7"/>
+      <c r="F14" s="7"/>
+      <c r="G14" s="7"/>
+      <c r="H14" s="7"/>
+      <c r="I14" s="7"/>
+      <c r="J14" s="7"/>
+      <c r="K14" s="7"/>
+      <c r="L14" s="7"/>
+      <c r="M14" s="7"/>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
@@ -20767,21 +20764,21 @@
       </c>
     </row>
     <row r="27" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A27" s="5" t="s">
+      <c r="A27" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="B27" s="5"/>
-      <c r="C27" s="5"/>
-      <c r="D27" s="5"/>
-      <c r="E27" s="5"/>
-      <c r="F27" s="5"/>
-      <c r="G27" s="5"/>
-      <c r="H27" s="5"/>
-      <c r="I27" s="5"/>
-      <c r="J27" s="5"/>
-      <c r="K27" s="5"/>
-      <c r="L27" s="5"/>
-      <c r="M27" s="5"/>
+      <c r="B27" s="7"/>
+      <c r="C27" s="7"/>
+      <c r="D27" s="7"/>
+      <c r="E27" s="7"/>
+      <c r="F27" s="7"/>
+      <c r="G27" s="7"/>
+      <c r="H27" s="7"/>
+      <c r="I27" s="7"/>
+      <c r="J27" s="7"/>
+      <c r="K27" s="7"/>
+      <c r="L27" s="7"/>
+      <c r="M27" s="7"/>
     </row>
     <row r="28" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A28" s="1" t="s">
@@ -21235,21 +21232,21 @@
       </c>
     </row>
     <row r="40" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A40" s="5" t="s">
+      <c r="A40" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="B40" s="5"/>
-      <c r="C40" s="5"/>
-      <c r="D40" s="5"/>
-      <c r="E40" s="5"/>
-      <c r="F40" s="5"/>
-      <c r="G40" s="5"/>
-      <c r="H40" s="5"/>
-      <c r="I40" s="5"/>
-      <c r="J40" s="5"/>
-      <c r="K40" s="5"/>
-      <c r="L40" s="5"/>
-      <c r="M40" s="5"/>
+      <c r="B40" s="7"/>
+      <c r="C40" s="7"/>
+      <c r="D40" s="7"/>
+      <c r="E40" s="7"/>
+      <c r="F40" s="7"/>
+      <c r="G40" s="7"/>
+      <c r="H40" s="7"/>
+      <c r="I40" s="7"/>
+      <c r="J40" s="7"/>
+      <c r="K40" s="7"/>
+      <c r="L40" s="7"/>
+      <c r="M40" s="7"/>
     </row>
     <row r="41" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A41" s="1" t="s">
@@ -21724,15 +21721,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="5"/>
-      <c r="C1" s="5"/>
-      <c r="D1" s="5"/>
-      <c r="E1" s="5"/>
-      <c r="F1" s="5"/>
-      <c r="G1" s="5"/>
+      <c r="B1" s="7"/>
+      <c r="C1" s="7"/>
+      <c r="D1" s="7"/>
+      <c r="E1" s="7"/>
+      <c r="F1" s="7"/>
+      <c r="G1" s="7"/>
     </row>
     <row r="2" spans="1:8" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
@@ -21945,15 +21942,15 @@
     </row>
     <row r="11" spans="1:8" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="12" spans="1:8" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="5" t="s">
+      <c r="A12" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="B12" s="5"/>
-      <c r="C12" s="5"/>
-      <c r="D12" s="5"/>
-      <c r="E12" s="5"/>
-      <c r="F12" s="5"/>
-      <c r="G12" s="5"/>
+      <c r="B12" s="7"/>
+      <c r="C12" s="7"/>
+      <c r="D12" s="7"/>
+      <c r="E12" s="7"/>
+      <c r="F12" s="7"/>
+      <c r="G12" s="7"/>
     </row>
     <row r="13" spans="1:8" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
@@ -22164,15 +22161,15 @@
     </row>
     <row r="22" spans="1:8" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="23" spans="1:8" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="5" t="s">
+      <c r="A23" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="B23" s="5"/>
-      <c r="C23" s="5"/>
-      <c r="D23" s="5"/>
-      <c r="E23" s="5"/>
-      <c r="F23" s="5"/>
-      <c r="G23" s="5"/>
+      <c r="B23" s="7"/>
+      <c r="C23" s="7"/>
+      <c r="D23" s="7"/>
+      <c r="E23" s="7"/>
+      <c r="F23" s="7"/>
+      <c r="G23" s="7"/>
     </row>
     <row r="24" spans="1:8" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
@@ -22385,15 +22382,15 @@
     </row>
     <row r="33" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="34" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="5" t="s">
+      <c r="A34" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="B34" s="5"/>
-      <c r="C34" s="5"/>
-      <c r="D34" s="5"/>
-      <c r="E34" s="5"/>
-      <c r="F34" s="5"/>
-      <c r="G34" s="5"/>
+      <c r="B34" s="7"/>
+      <c r="C34" s="7"/>
+      <c r="D34" s="7"/>
+      <c r="E34" s="7"/>
+      <c r="F34" s="7"/>
+      <c r="G34" s="7"/>
     </row>
     <row r="35" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="1" t="s">
@@ -36103,7 +36100,7 @@
     <col min="9" max="9" width="8.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>106</v>
       </c>
@@ -36114,7 +36111,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>94</v>
       </c>
@@ -36146,7 +36143,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
         <v>1</v>
       </c>
@@ -36177,8 +36174,16 @@
       <c r="J3" s="1">
         <v>8</v>
       </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K3">
+        <f>I3/100</f>
+        <v>0.03</v>
+      </c>
+      <c r="L3">
+        <f>(POWER(1.022,A3))+8*A3</f>
+        <v>9.0220000000000002</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
         <v>2</v>
       </c>
@@ -36209,8 +36214,16 @@
       <c r="J4" s="1">
         <v>16</v>
       </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K4">
+        <f>(I4-I3)/100</f>
+        <v>0.02</v>
+      </c>
+      <c r="L4">
+        <f t="shared" ref="L4:L22" si="0">(POWER(1.022,A4))+8*A4</f>
+        <v>17.044484000000001</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A5" s="1">
         <v>3</v>
       </c>
@@ -36241,8 +36254,16 @@
       <c r="J5" s="1">
         <v>24</v>
       </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K5">
+        <f t="shared" ref="K5:K22" si="1">(I5-I4)/100</f>
+        <v>0.03</v>
+      </c>
+      <c r="L5">
+        <f t="shared" si="0"/>
+        <v>25.067462647999999</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A6" s="1">
         <v>4</v>
       </c>
@@ -36273,8 +36294,16 @@
       <c r="J6" s="1">
         <v>32</v>
       </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K6">
+        <f t="shared" si="1"/>
+        <v>0.02</v>
+      </c>
+      <c r="L6">
+        <f t="shared" si="0"/>
+        <v>33.090946826256001</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A7" s="1">
         <v>5</v>
       </c>
@@ -36305,8 +36334,16 @@
       <c r="J7" s="1">
         <v>40</v>
       </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K7">
+        <f t="shared" si="1"/>
+        <v>0.03</v>
+      </c>
+      <c r="L7">
+        <f t="shared" si="0"/>
+        <v>41.114947656433635</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A8" s="1">
         <v>6</v>
       </c>
@@ -36337,8 +36374,16 @@
       <c r="J8" s="1">
         <v>48</v>
       </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K8">
+        <f t="shared" si="1"/>
+        <v>0.03</v>
+      </c>
+      <c r="L8">
+        <f t="shared" si="0"/>
+        <v>49.139476504875169</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A9" s="1">
         <v>7</v>
       </c>
@@ -36369,8 +36414,16 @@
       <c r="J9" s="1">
         <v>56</v>
       </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K9">
+        <f t="shared" si="1"/>
+        <v>0.03</v>
+      </c>
+      <c r="L9">
+        <f t="shared" si="0"/>
+        <v>57.164544987982424</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A10" s="1">
         <v>8</v>
       </c>
@@ -36401,8 +36454,16 @@
       <c r="J10" s="1">
         <v>64</v>
       </c>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K10">
+        <f t="shared" si="1"/>
+        <v>0.03</v>
+      </c>
+      <c r="L10">
+        <f t="shared" si="0"/>
+        <v>65.190164977718041</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A11" s="1">
         <v>9</v>
       </c>
@@ -36433,8 +36494,16 @@
       <c r="J11" s="1">
         <v>72</v>
       </c>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K11">
+        <f t="shared" si="1"/>
+        <v>0.03</v>
+      </c>
+      <c r="L11">
+        <f t="shared" si="0"/>
+        <v>73.216348607227843</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A12" s="1">
         <v>10</v>
       </c>
@@ -36465,8 +36534,16 @@
       <c r="J12" s="1">
         <v>80</v>
       </c>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K12">
+        <f t="shared" si="1"/>
+        <v>0.03</v>
+      </c>
+      <c r="L12">
+        <f t="shared" si="0"/>
+        <v>81.243108276586852</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A13" s="1">
         <v>11</v>
       </c>
@@ -36497,8 +36574,16 @@
       <c r="J13" s="1">
         <v>88</v>
       </c>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K13">
+        <f t="shared" si="1"/>
+        <v>0.03</v>
+      </c>
+      <c r="L13">
+        <f t="shared" si="0"/>
+        <v>89.270456658671762</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A14" s="1">
         <v>12</v>
       </c>
@@ -36529,8 +36614,16 @@
       <c r="J14" s="1">
         <v>96</v>
       </c>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K14">
+        <f t="shared" si="1"/>
+        <v>0.04</v>
+      </c>
+      <c r="L14">
+        <f t="shared" si="0"/>
+        <v>97.298406705162535</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A15" s="1">
         <v>13</v>
       </c>
@@ -36561,8 +36654,16 @@
       <c r="J15" s="1">
         <v>104</v>
       </c>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K15">
+        <f t="shared" si="1"/>
+        <v>0.03</v>
+      </c>
+      <c r="L15">
+        <f t="shared" si="0"/>
+        <v>105.32697165267611</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A16" s="1">
         <v>14</v>
       </c>
@@ -36593,8 +36694,16 @@
       <c r="J16" s="1">
         <v>112</v>
       </c>
-    </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K16">
+        <f t="shared" si="1"/>
+        <v>0.03</v>
+      </c>
+      <c r="L16">
+        <f t="shared" si="0"/>
+        <v>113.35616502903498</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A17" s="1">
         <v>15</v>
       </c>
@@ -36625,8 +36734,16 @@
       <c r="J17" s="1">
         <v>120</v>
       </c>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K17">
+        <f t="shared" si="1"/>
+        <v>0.04</v>
+      </c>
+      <c r="L17">
+        <f t="shared" si="0"/>
+        <v>121.38600065967375</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A18" s="1">
         <v>16</v>
       </c>
@@ -36657,8 +36774,16 @@
       <c r="J18" s="1">
         <v>128</v>
       </c>
-    </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K18">
+        <f t="shared" si="1"/>
+        <v>0.04</v>
+      </c>
+      <c r="L18">
+        <f t="shared" si="0"/>
+        <v>129.41649267418657</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A19" s="1">
         <v>17</v>
       </c>
@@ -36689,8 +36814,16 @@
       <c r="J19" s="1">
         <v>136</v>
       </c>
-    </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K19">
+        <f t="shared" si="1"/>
+        <v>0.03</v>
+      </c>
+      <c r="L19">
+        <f t="shared" si="0"/>
+        <v>137.44765551301867</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A20" s="1">
         <v>18</v>
       </c>
@@ -36721,8 +36854,16 @@
       <c r="J20" s="1">
         <v>144</v>
       </c>
-    </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K20">
+        <f t="shared" si="1"/>
+        <v>0.04</v>
+      </c>
+      <c r="L20">
+        <f t="shared" si="0"/>
+        <v>145.47950393430509</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A21" s="1">
         <v>19</v>
       </c>
@@ -36753,8 +36894,16 @@
       <c r="J21" s="1">
         <v>152</v>
       </c>
-    </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K21">
+        <f t="shared" si="1"/>
+        <v>0.04</v>
+      </c>
+      <c r="L21">
+        <f t="shared" si="0"/>
+        <v>153.51205302085981</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A22" s="1">
         <v>20</v>
       </c>
@@ -36785,8 +36934,16 @@
       <c r="J22" s="1">
         <v>160</v>
       </c>
-    </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K22">
+        <f t="shared" si="1"/>
+        <v>0.04</v>
+      </c>
+      <c r="L22">
+        <f t="shared" si="0"/>
+        <v>161.54531818731871</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A23" s="1"/>
       <c r="B23" s="1"/>
       <c r="C23" s="1"/>
@@ -36797,7 +36954,7 @@
       <c r="H23" s="3"/>
       <c r="I23" s="1"/>
     </row>
-    <row r="24" spans="1:10" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:12" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>97</v>
       </c>
@@ -36808,7 +36965,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="25" spans="1:10" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:12" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>94</v>
       </c>
@@ -36840,7 +36997,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="26" spans="1:10" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:12" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="1">
         <v>1</v>
       </c>
@@ -36871,8 +37028,12 @@
       <c r="J26" s="1">
         <v>6</v>
       </c>
-    </row>
-    <row r="27" spans="1:10" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="L26">
+        <f>POWER(1.026,A26)+5</f>
+        <v>6.0259999999999998</v>
+      </c>
+    </row>
+    <row r="27" spans="1:12" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="1">
         <v>2</v>
       </c>
@@ -36903,8 +37064,12 @@
       <c r="J27" s="1">
         <v>12</v>
       </c>
-    </row>
-    <row r="28" spans="1:10" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="L27">
+        <f>A27*$L$26</f>
+        <v>12.052</v>
+      </c>
+    </row>
+    <row r="28" spans="1:12" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="1">
         <v>3</v>
       </c>
@@ -36935,8 +37100,12 @@
       <c r="J28" s="1">
         <v>18</v>
       </c>
-    </row>
-    <row r="29" spans="1:10" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="L28">
+        <f t="shared" ref="L28:L45" si="2">A28*$L$26</f>
+        <v>18.077999999999999</v>
+      </c>
+    </row>
+    <row r="29" spans="1:12" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="1">
         <v>4</v>
       </c>
@@ -36967,8 +37136,12 @@
       <c r="J29" s="1">
         <v>24</v>
       </c>
-    </row>
-    <row r="30" spans="1:10" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="L29">
+        <f t="shared" si="2"/>
+        <v>24.103999999999999</v>
+      </c>
+    </row>
+    <row r="30" spans="1:12" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="1">
         <v>5</v>
       </c>
@@ -36999,8 +37172,12 @@
       <c r="J30" s="1">
         <v>30</v>
       </c>
-    </row>
-    <row r="31" spans="1:10" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="L30">
+        <f t="shared" si="2"/>
+        <v>30.13</v>
+      </c>
+    </row>
+    <row r="31" spans="1:12" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="1">
         <v>6</v>
       </c>
@@ -37031,8 +37208,12 @@
       <c r="J31" s="1">
         <v>36</v>
       </c>
-    </row>
-    <row r="32" spans="1:10" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="L31">
+        <f t="shared" si="2"/>
+        <v>36.155999999999999</v>
+      </c>
+    </row>
+    <row r="32" spans="1:12" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="1">
         <v>7</v>
       </c>
@@ -37063,8 +37244,12 @@
       <c r="J32" s="1">
         <v>42</v>
       </c>
-    </row>
-    <row r="33" spans="1:10" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="L32">
+        <f t="shared" si="2"/>
+        <v>42.182000000000002</v>
+      </c>
+    </row>
+    <row r="33" spans="1:12" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="1">
         <v>8</v>
       </c>
@@ -37095,8 +37280,12 @@
       <c r="J33" s="1">
         <v>48</v>
       </c>
-    </row>
-    <row r="34" spans="1:10" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="L33">
+        <f t="shared" si="2"/>
+        <v>48.207999999999998</v>
+      </c>
+    </row>
+    <row r="34" spans="1:12" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="1">
         <v>9</v>
       </c>
@@ -37127,8 +37316,12 @@
       <c r="J34" s="1">
         <v>54</v>
       </c>
-    </row>
-    <row r="35" spans="1:10" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="L34">
+        <f t="shared" si="2"/>
+        <v>54.233999999999995</v>
+      </c>
+    </row>
+    <row r="35" spans="1:12" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="1">
         <v>10</v>
       </c>
@@ -37159,8 +37352,12 @@
       <c r="J35" s="1">
         <v>60</v>
       </c>
-    </row>
-    <row r="36" spans="1:10" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="L35">
+        <f t="shared" si="2"/>
+        <v>60.26</v>
+      </c>
+    </row>
+    <row r="36" spans="1:12" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="1">
         <v>11</v>
       </c>
@@ -37191,8 +37388,12 @@
       <c r="J36" s="1">
         <v>66</v>
       </c>
-    </row>
-    <row r="37" spans="1:10" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="L36">
+        <f t="shared" si="2"/>
+        <v>66.286000000000001</v>
+      </c>
+    </row>
+    <row r="37" spans="1:12" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" s="1">
         <v>12</v>
       </c>
@@ -37223,8 +37424,12 @@
       <c r="J37" s="1">
         <v>72</v>
       </c>
-    </row>
-    <row r="38" spans="1:10" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="L37">
+        <f t="shared" si="2"/>
+        <v>72.311999999999998</v>
+      </c>
+    </row>
+    <row r="38" spans="1:12" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="1">
         <v>13</v>
       </c>
@@ -37255,8 +37460,12 @@
       <c r="J38" s="1">
         <v>78</v>
       </c>
-    </row>
-    <row r="39" spans="1:10" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="L38">
+        <f t="shared" si="2"/>
+        <v>78.337999999999994</v>
+      </c>
+    </row>
+    <row r="39" spans="1:12" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="1">
         <v>14</v>
       </c>
@@ -37287,8 +37496,12 @@
       <c r="J39" s="1">
         <v>84</v>
       </c>
-    </row>
-    <row r="40" spans="1:10" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="L39">
+        <f t="shared" si="2"/>
+        <v>84.364000000000004</v>
+      </c>
+    </row>
+    <row r="40" spans="1:12" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="1">
         <v>15</v>
       </c>
@@ -37319,8 +37532,12 @@
       <c r="J40" s="1">
         <v>90</v>
       </c>
-    </row>
-    <row r="41" spans="1:10" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="L40">
+        <f t="shared" si="2"/>
+        <v>90.39</v>
+      </c>
+    </row>
+    <row r="41" spans="1:12" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41" s="1">
         <v>16</v>
       </c>
@@ -37351,8 +37568,12 @@
       <c r="J41" s="1">
         <v>96</v>
       </c>
-    </row>
-    <row r="42" spans="1:10" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="L41">
+        <f t="shared" si="2"/>
+        <v>96.415999999999997</v>
+      </c>
+    </row>
+    <row r="42" spans="1:12" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" s="1">
         <v>17</v>
       </c>
@@ -37383,8 +37604,12 @@
       <c r="J42" s="1">
         <v>102</v>
       </c>
-    </row>
-    <row r="43" spans="1:10" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="L42">
+        <f t="shared" si="2"/>
+        <v>102.44199999999999</v>
+      </c>
+    </row>
+    <row r="43" spans="1:12" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A43" s="1">
         <v>18</v>
       </c>
@@ -37415,8 +37640,12 @@
       <c r="J43" s="1">
         <v>108</v>
       </c>
-    </row>
-    <row r="44" spans="1:10" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="L43">
+        <f t="shared" si="2"/>
+        <v>108.46799999999999</v>
+      </c>
+    </row>
+    <row r="44" spans="1:12" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A44" s="1">
         <v>19</v>
       </c>
@@ -37447,8 +37676,12 @@
       <c r="J44" s="1">
         <v>114</v>
       </c>
-    </row>
-    <row r="45" spans="1:10" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="L44">
+        <f t="shared" si="2"/>
+        <v>114.494</v>
+      </c>
+    </row>
+    <row r="45" spans="1:12" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A45" s="1">
         <v>20</v>
       </c>
@@ -37479,8 +37712,12 @@
       <c r="J45" s="1">
         <v>120</v>
       </c>
-    </row>
-    <row r="46" spans="1:10" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="L45">
+        <f t="shared" si="2"/>
+        <v>120.52</v>
+      </c>
+    </row>
+    <row r="46" spans="1:12" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A46" s="1"/>
       <c r="B46" s="1"/>
       <c r="C46" s="1"/>
@@ -37491,7 +37728,7 @@
       <c r="H46" s="3"/>
       <c r="I46" s="1"/>
     </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>92</v>
       </c>
@@ -38179,7 +38416,7 @@
       <c r="H73" s="3">
         <v>2.3148148148148147E-2</v>
       </c>
-      <c r="I73" s="8">
+      <c r="I73" s="1">
         <v>0.05</v>
       </c>
     </row>
@@ -38208,7 +38445,7 @@
       <c r="H74" s="3">
         <v>3.0324074074074073E-2</v>
       </c>
-      <c r="I74" s="8">
+      <c r="I74" s="1">
         <v>0.1</v>
       </c>
     </row>
@@ -38237,7 +38474,7 @@
       <c r="H75" s="3">
         <v>3.8657407407407404E-2</v>
       </c>
-      <c r="I75" s="8">
+      <c r="I75" s="1">
         <v>0.15</v>
       </c>
     </row>
@@ -38266,7 +38503,7 @@
       <c r="H76" s="3">
         <v>4.8263888888888891E-2</v>
       </c>
-      <c r="I76" s="8">
+      <c r="I76" s="1">
         <v>0.2</v>
       </c>
     </row>
@@ -38295,7 +38532,7 @@
       <c r="H77" s="3">
         <v>5.949074074074074E-2</v>
       </c>
-      <c r="I77" s="8">
+      <c r="I77" s="1">
         <v>0.25</v>
       </c>
     </row>
@@ -38324,7 +38561,7 @@
       <c r="H78" s="3">
         <v>7.2453703703703701E-2</v>
       </c>
-      <c r="I78" s="8">
+      <c r="I78" s="1">
         <v>0.3</v>
       </c>
     </row>
@@ -38353,7 +38590,7 @@
       <c r="H79" s="3">
         <v>8.7615740740740744E-2</v>
       </c>
-      <c r="I79" s="8">
+      <c r="I79" s="1">
         <v>0.35</v>
       </c>
     </row>
@@ -38382,7 +38619,7 @@
       <c r="H80" s="3">
         <v>0.1050925925925926</v>
       </c>
-      <c r="I80" s="8">
+      <c r="I80" s="1">
         <v>0.4</v>
       </c>
     </row>
@@ -38411,7 +38648,7 @@
       <c r="H81" s="3">
         <v>0.12534722222222222</v>
       </c>
-      <c r="I81" s="8">
+      <c r="I81" s="1">
         <v>0.45</v>
       </c>
     </row>
@@ -38440,7 +38677,7 @@
       <c r="H82" s="3">
         <v>0.14884259259259258</v>
       </c>
-      <c r="I82" s="8">
+      <c r="I82" s="1">
         <v>0.5</v>
       </c>
     </row>
@@ -38469,7 +38706,7 @@
       <c r="H83" s="3">
         <v>0.1761574074074074</v>
       </c>
-      <c r="I83" s="8">
+      <c r="I83" s="1">
         <v>0.55000000000000004</v>
       </c>
     </row>
@@ -38498,7 +38735,7 @@
       <c r="H84" s="3">
         <v>0.20775462962962962</v>
       </c>
-      <c r="I84" s="8">
+      <c r="I84" s="1">
         <v>0.6</v>
       </c>
     </row>
@@ -38527,7 +38764,7 @@
       <c r="H85" s="3">
         <v>0.24456018518518519</v>
       </c>
-      <c r="I85" s="8">
+      <c r="I85" s="1">
         <v>0.65</v>
       </c>
     </row>
@@ -38556,7 +38793,7 @@
       <c r="H86" s="3">
         <v>0.28715277777777776</v>
       </c>
-      <c r="I86" s="8">
+      <c r="I86" s="1">
         <v>0.7</v>
       </c>
     </row>
@@ -38585,7 +38822,7 @@
       <c r="H87" s="3">
         <v>0.33657407407407408</v>
       </c>
-      <c r="I87" s="8">
+      <c r="I87" s="1">
         <v>0.75</v>
       </c>
     </row>
@@ -38614,7 +38851,7 @@
       <c r="H88" s="3">
         <v>0.39386574074074077</v>
       </c>
-      <c r="I88" s="8">
+      <c r="I88" s="1">
         <v>0.8</v>
       </c>
     </row>
@@ -38643,7 +38880,7 @@
       <c r="H89" s="3">
         <v>0.46030092592592592</v>
       </c>
-      <c r="I89" s="8">
+      <c r="I89" s="1">
         <v>0.85</v>
       </c>
     </row>
@@ -38672,7 +38909,7 @@
       <c r="H90" s="3">
         <v>0.53749999999999998</v>
       </c>
-      <c r="I90" s="8">
+      <c r="I90" s="1">
         <v>0.9</v>
       </c>
     </row>
@@ -38701,7 +38938,7 @@
       <c r="H91" s="3">
         <v>0.6269675925925926</v>
       </c>
-      <c r="I91" s="8">
+      <c r="I91" s="1">
         <v>0.95</v>
       </c>
     </row>
@@ -38730,7 +38967,7 @@
       <c r="H92" s="3">
         <v>0.73067129629629635</v>
       </c>
-      <c r="I92" s="8">
+      <c r="I92" s="1">
         <v>1</v>
       </c>
     </row>
@@ -39422,7 +39659,7 @@
       <c r="H119" s="2">
         <v>2.3148148148148147E-2</v>
       </c>
-      <c r="I119" s="7">
+      <c r="I119" s="6">
         <v>2</v>
       </c>
       <c r="J119" s="1">
@@ -39454,7 +39691,7 @@
       <c r="H120" s="2">
         <v>3.0324074074074073E-2</v>
       </c>
-      <c r="I120" s="7">
+      <c r="I120" s="6">
         <v>4</v>
       </c>
       <c r="J120" s="1">
@@ -39486,7 +39723,7 @@
       <c r="H121" s="2">
         <v>3.8657407407407404E-2</v>
       </c>
-      <c r="I121" s="7">
+      <c r="I121" s="6">
         <v>6</v>
       </c>
       <c r="J121" s="1">
@@ -39518,7 +39755,7 @@
       <c r="H122" s="2">
         <v>4.8263888888888891E-2</v>
       </c>
-      <c r="I122" s="7">
+      <c r="I122" s="6">
         <v>4</v>
       </c>
       <c r="J122" s="1">
@@ -39550,7 +39787,7 @@
       <c r="H123" s="2">
         <v>5.949074074074074E-2</v>
       </c>
-      <c r="I123" s="7">
+      <c r="I123" s="6">
         <v>10</v>
       </c>
       <c r="J123" s="1">
@@ -39582,7 +39819,7 @@
       <c r="H124" s="2">
         <v>7.2453703703703701E-2</v>
       </c>
-      <c r="I124" s="7">
+      <c r="I124" s="6">
         <v>13</v>
       </c>
       <c r="J124" s="1">
@@ -39614,7 +39851,7 @@
       <c r="H125" s="2">
         <v>8.7615740740740744E-2</v>
       </c>
-      <c r="I125" s="7">
+      <c r="I125" s="6">
         <v>15</v>
       </c>
       <c r="J125" s="1">
@@ -39646,7 +39883,7 @@
       <c r="H126" s="2">
         <v>0.1050925925925926</v>
       </c>
-      <c r="I126" s="7">
+      <c r="I126" s="6">
         <v>17</v>
       </c>
       <c r="J126" s="1">
@@ -39679,13 +39916,13 @@
       <c r="H127" s="2">
         <v>0.12534722222222222</v>
       </c>
-      <c r="I127" s="7">
+      <c r="I127" s="6">
         <v>18</v>
       </c>
       <c r="J127" s="1">
         <v>90</v>
       </c>
-      <c r="M127" s="6"/>
+      <c r="M127" s="5"/>
     </row>
     <row r="128" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A128" s="1">
@@ -39712,7 +39949,7 @@
       <c r="H128" s="2">
         <v>0.14884259259259258</v>
       </c>
-      <c r="I128" s="7">
+      <c r="I128" s="6">
         <v>22</v>
       </c>
       <c r="J128" s="1">
@@ -39744,7 +39981,7 @@
       <c r="H129" s="2">
         <v>0.1761574074074074</v>
       </c>
-      <c r="I129" s="7">
+      <c r="I129" s="6">
         <v>24</v>
       </c>
       <c r="J129" s="1">
@@ -39776,7 +40013,7 @@
       <c r="H130" s="2">
         <v>0.20775462962962962</v>
       </c>
-      <c r="I130" s="7">
+      <c r="I130" s="6">
         <v>27</v>
       </c>
       <c r="J130" s="1">
@@ -39808,7 +40045,7 @@
       <c r="H131" s="2">
         <v>0.24456018518518519</v>
       </c>
-      <c r="I131" s="7">
+      <c r="I131" s="6">
         <v>29</v>
       </c>
       <c r="J131" s="1">
@@ -39840,7 +40077,7 @@
       <c r="H132" s="2">
         <v>0.28715277777777776</v>
       </c>
-      <c r="I132" s="7">
+      <c r="I132" s="6">
         <v>32</v>
       </c>
       <c r="J132" s="1">
@@ -39872,7 +40109,7 @@
       <c r="H133" s="2">
         <v>0.33657407407407408</v>
       </c>
-      <c r="I133" s="7">
+      <c r="I133" s="6">
         <v>35</v>
       </c>
       <c r="J133" s="1">
@@ -39904,7 +40141,7 @@
       <c r="H134" s="2">
         <v>0.39386574074074077</v>
       </c>
-      <c r="I134" s="7">
+      <c r="I134" s="6">
         <v>37</v>
       </c>
       <c r="J134" s="1">
@@ -39936,7 +40173,7 @@
       <c r="H135" s="2">
         <v>0.46030092592592592</v>
       </c>
-      <c r="I135" s="7">
+      <c r="I135" s="6">
         <v>40</v>
       </c>
       <c r="J135" s="1">
@@ -39968,7 +40205,7 @@
       <c r="H136" s="2">
         <v>0.53749999999999998</v>
       </c>
-      <c r="I136" s="7">
+      <c r="I136" s="6">
         <v>43</v>
       </c>
       <c r="J136" s="1">
@@ -40000,7 +40237,7 @@
       <c r="H137" s="2">
         <v>0.6269675925925926</v>
       </c>
-      <c r="I137" s="7">
+      <c r="I137" s="6">
         <v>46</v>
       </c>
       <c r="J137" s="1">
@@ -40032,7 +40269,7 @@
       <c r="H138" s="2">
         <v>0.73067129629629635</v>
       </c>
-      <c r="I138" s="7">
+      <c r="I138" s="6">
         <v>49</v>
       </c>
       <c r="J138" s="1">

</xml_diff>